<commit_message>
Add second invoice (No. 21) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="الفاتورة" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="فاتورة 25-06" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="فاتورة 21" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +470,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
@@ -484,7 +485,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>فاتورة رقم:</t>
+          <t>فاتورة رقم: -</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -892,6 +893,455 @@
       <c r="D22" s="7" t="inlineStr">
         <is>
           <t>6360,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 21</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 27/06/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>485,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1455,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>حلبة</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>كلانس أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>جام أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>ألمنيوم كيس</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>كلانس 24</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>سربت</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>كلنكس</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي علبة جوخ كبير</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي علبة فلافل</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي شوربة عربي</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي علبة فتوش</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>295,00</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>295,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>مسطرة</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>15,00</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>5600,00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct merchandise names in invoice No. 21 sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>حلبة</t>
+          <t>حلبت</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>كلانس 24</t>
+          <t>كلانش 24</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>سربت</t>
+          <t>سربيت</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Update invoice No. 21 item names per user-provided list
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -965,7 +965,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>النشا</t>
+          <t>ليباي</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>ملعقة</t>
+          <t>كوفرتة أ مبرطمي</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>الزيت</t>
+          <t>كلينكس عادي</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>سربت</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>علبة</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>الطوب</t>
+          <t>زيتون</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>كلانس أ مبرطمي</t>
+          <t>علبة صغيرة</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>جام أ مبرطمي</t>
+          <t>البنط</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>ألمنيوم كيس</t>
+          <t>الطماطم عائشة</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>كلانش 24</t>
+          <t>جام أ مبرطمي</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>سربيت</t>
+          <t>الصندوق أكاجو</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>كلنكس</t>
+          <t>اللون البلدي</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>أمبرطمي علبة جوخ كبير</t>
+          <t>فلفل مدخن</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>أمبرطمي علبة فلافل</t>
+          <t>كرطون الثوم</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>أمبرطمي شوربة عربي</t>
+          <t>كبسون</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>أمبرطمي علبة فتوش</t>
+          <t>حافظ</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>مسطرة</t>
+          <t>سلوفان (900m)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Finalize invoice No. 21 item names
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -965,7 +965,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>ليباي</t>
+          <t>النشا</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>كوفرتة أ مبرطمي</t>
+          <t>ملعقة</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>كلينكس عادي</t>
+          <t>الزيت</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>سربت</t>
+          <t>حلبت</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>علبة</t>
+          <t>زيتون</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>الطوب</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>علبة صغيرة</t>
+          <t>كلانس أ مبرطمي</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>البنط</t>
+          <t>جام أ مبرطمي</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>الطماطم عائشة</t>
+          <t>ألمنيوم كيس</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>جام أ مبرطمي</t>
+          <t>كلانش 24</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>الصندوق أكاجو</t>
+          <t>سربيت</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>اللون البلدي</t>
+          <t>كلنكس</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>فلفل مدخن</t>
+          <t>أمبرطمي علبة جوخ كبير</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>كرطون الثوم</t>
+          <t>أمبرطمي علبة فلافل</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>كبسون</t>
+          <t>أمبرطمي شوربة عربي</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>حافظ</t>
+          <t>أمبرطمي علبة فتوش</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>سلوفان (900m)</t>
+          <t>مسطرة</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add invoices No. 23, 94, and 24 as separate sheets
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="فاتورة 25-06" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="فاتورة 21" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="فاتورة 23" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="فاتورة 94" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="فاتورة 24" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,8 +472,8 @@
   <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
@@ -910,8 +913,8 @@
   <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1348,4 +1351,1615 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 23</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 28/06/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>485,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1455,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>قندري</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>كبسون</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>175,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>175,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>نسمة 2K</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>جام أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>كنور دجاج</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>فرقوم غلانط</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>22,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>44,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>سلوفان كيس</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>336,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>كلانش سطاريط</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>مسطرة 2K</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>38,00</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>228,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>كونيس أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>أ مبرطمي نصف كيلو</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>علبة جوخ تونسي</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>ثوم بودر + بصل بودر</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>60,00</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>5573,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 94</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 29/06/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>485,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1940,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>نسمة 2K</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>114,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>كلانش أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>قلاي 100</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>مملكة الزبل</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>كلنكس عادي</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي شوربة عربي</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>الشوب مسوس 2K</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>225,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>سكر</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>6,50</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>سكر أزريقة</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>7,00</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>الشاي</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>حمص 2K</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>750,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>غيار طاولة</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>312,00</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>1248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي بواط صوف</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>430,00</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>430,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>8035,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 24</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 30/06/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>485,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1455,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>نسمة 2K</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>كنور الدجاج</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>6K</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>بسكويت كبيرة</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>40,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>كلانش 24</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>كنور 10K</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>104,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي هريسة كومة ولبن حليب</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي علبة فلافل</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي نصف كيلو</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>بكية حقائب</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>400,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي شطل كريسي</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>1050,00</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>1050,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>3K</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>الثوم</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>5909,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add corrected invoice No. 24 (01/07) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -12,6 +12,7 @@
     <sheet name="فاتورة 23" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="فاتورة 94" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="فاتورة 24" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="فاتورة 24 (1-07)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2962,4 +2963,387 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 24</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 01/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>485,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1940,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>كلانش أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>جام أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>كوفرتة أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>سربت</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>كرطون أ مبرطمي علبة محلبية</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>كرطون</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>مسكة اللاصقة</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>40,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي ألمنيوم نصف كيلو</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>900,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>900,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>5787,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add invoice No. 25 (03/07) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -13,6 +13,7 @@
     <sheet name="فاتورة 94" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="فاتورة 24" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فاتورة 24 (1-07)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="فاتورة 25" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3346,4 +3347,519 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 25</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 03/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>40,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>ليكات</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>عدس أحمر</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>18,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>بنزاي</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>90,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>270,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>كرطون الدرش حامين</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>265,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>265,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>السفنا</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>114,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>336,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي شوربة عربي</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي صوجي كيس تونسية</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>576,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>كرطون بنزا كيس</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>88,00</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>440,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>كوبايلي</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>0,35</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>210,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>FAX لبكسر SL</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>مسطرة VMA 2K</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>38,00</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>228,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>6527,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add invoice No. 26 (04/07) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -14,6 +14,7 @@
     <sheet name="فاتورة 24" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="فاتورة 24 (1-07)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="فاتورة 25" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="فاتورة 26" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3862,4 +3863,563 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 26</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 04/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>كنور</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>156,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>كلانش بسكري كبيرة</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>22,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>132,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>سكر أبيض</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>6,50</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>سكر أزريقة</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>7,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>ليكات</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>بنزاي أبيض</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>280,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>576,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>كلانكس حام كيس</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>352,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>352,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي علبة فلافل</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي طبوصي تونسية ولبن</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي شوربة عربي بلبن</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي كوفس</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي علبة صوجي تونسية</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>جام أمبرطمي + كلانش أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>480,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>غيار طاولة</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>312,00</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>936,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>9001,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add invoice No. 26 (05/07) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -15,6 +15,7 @@
     <sheet name="فاتورة 24 (1-07)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="فاتورة 25" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="فاتورة 26" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="فاتورة 26 (5-07)" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4422,4 +4423,431 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 26</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 05/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>كوفس أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>ألمنيوم</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>510,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>سلوفان</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>خل أبيض</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>8,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>96,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>كرطون زنجبيل</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>كرطون شوكة</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>390,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>780,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>5640,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add invoice dated 06/07 as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -16,6 +16,7 @@
     <sheet name="فاتورة 25" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="فاتورة 26" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="فاتورة 26 (5-07)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="فاتورة 6-07" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -908,6 +909,279 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: -</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 06/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>جام أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>كلانش أمبرطمي</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>كلانش 24</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>22,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>132,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>الشاي</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>2729,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 27 (08/07) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -17,6 +17,7 @@
     <sheet name="فاتورة 26" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="فاتورة 26 (5-07)" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="فاتورة 6-07" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="فاتورة 27" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1182,6 +1183,389 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 27</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 08/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>940,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>كلانش Star</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>310,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>كلانش أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>جام أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>منستون مقطع</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>65,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>195,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>كرطون عربي</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>3627,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 28 (10/07) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -18,6 +18,7 @@
     <sheet name="فاتورة 26 (5-07)" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="فاتورة 6-07" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="فاتورة 27" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="فاتورة 28" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1566,6 +1567,411 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 28</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 10/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>الزيت كرطون 5L</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>310,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>محسي صحو</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>ألمنيوم</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>510,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>مسكة الزبل</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>جام أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>كبسون أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>الهرسة صحا علبة كنانة</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>ليباي العجني</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي صحو مسوس نك العربي</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>4672,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice dated 11/07 as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -19,6 +19,7 @@
     <sheet name="فاتورة 6-07" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="فاتورة 27" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="فاتورة 28" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="فاتورة 11-07" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1972,6 +1973,389 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: -</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 11/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>كلانش Star</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>كنور</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>156,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>الطحين قندري 25</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>الشاي</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>4K</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>قرنون مقطوع بيض</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>4K</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>بنزا مقطوع مسوس</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>560,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>كنطون أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>4284,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 29 (12/07) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -20,6 +20,7 @@
     <sheet name="فاتورة 27" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="فاتورة 28" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="فاتورة 11-07" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="فاتورة 29" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2356,6 +2357,367 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 29</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 12/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>كلانش أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>جام أ مبرطمي</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>بنزا أسود</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>90,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>40,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>114,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>شطابة بالعصي</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>24,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>3746,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoices No. 29 (13/07), No. 30 (14/07), and 18/07
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -21,6 +21,9 @@
     <sheet name="فاتورة 28" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="فاتورة 11-07" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="فاتورة 29" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="فاتورة 29 (13-07)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="فاتورة 30" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="فاتورة 18-07" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2718,6 +2721,1529 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 29</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 13/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطمي شوربة عربي</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>بواط جوخ</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>13,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>130,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطي روتوس</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>كلانكس حام</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>كلانش Star</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>قرنون مقطوع</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>زنجبيل</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>كنور الدجاج</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>بنزا سنون 3K</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>255,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>كبسون 25</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>بوز غزال</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>480,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>نسبومحة</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>195,00</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>195,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>كلانش طابة</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>15,00</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>غيار طاولة</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>26,00</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>624,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>لبيه</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>7267,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 30</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 14/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>336,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>بكية جكفة سلك حريري</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>5,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>نسمة 25</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>حرقوم عياش</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>60,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>114,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>لوبي</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>كرطون زنجبيل</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>سلوفان</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>اللوبية</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>حمص</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>15,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>750,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>كلانش أ مبرطي</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>أمبرطي علب جوخ تونسية</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>علب كنانة</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>شطابة بالعصي</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>6456,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 9999721</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 18/07/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>جام أ مبرطي</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>كلانش أ مبرطي</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>سربيت NAYA</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>420,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>سكر أزريقة</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>7,00</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>سلوفان</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>قلاي</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>مسكة الزبل</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>كنور الدجاج</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>كرطون</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>425,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>4675,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Fix invoice No. 30 total (6476.50) and add invoice No. 44 (01/08)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -24,6 +24,7 @@
     <sheet name="فاتورة 29 (13-07)" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="فاتورة 30" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="فاتورة 18-07" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="فاتورة 44" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -71,7 +72,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -93,11 +94,17 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -114,6 +121,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3830,7 +3846,7 @@
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>6456,50</t>
+          <t>6476,50</t>
         </is>
       </c>
     </row>
@@ -4244,6 +4260,519 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 44</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 01/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>310,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>السكر أصفر</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>كنور</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>سلوفان</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>مسكة الزبل</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>420,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي شوربة عربي</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>كوفس أمبرطي</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي كنانة</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي روتوس</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي علب لبيه خيار</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>كوردون مغلف</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>29,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>290,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>6531,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. U1 (02/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -25,6 +25,7 @@
     <sheet name="فاتورة 30" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="فاتورة 18-07" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="فاتورة 44" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="فاتورة U1 (02-08)" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4773,6 +4774,515 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: U1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 02/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>315,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>نسمة 2K</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>كلانش Star 24</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>940,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>114,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>قرفة عواد</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>بطلة بودرة</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>60,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>يودمة بودرة</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>60,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>3+3</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>كلانش + جام أمبرطي</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>480,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>حلانة جلاك</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>10,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>البنزا سنون 2K3</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>255,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>الطوب 2K</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>اللوز أبعلي</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>130,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>260,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>كرطون الزنجبيل</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr"/>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>إضافي (كوكاز؟)</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>4582,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. U1 (03/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -26,6 +26,7 @@
     <sheet name="فاتورة 18-07" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="فاتورة 44" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="فاتورة U1 (02-08)" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="فاتورة U1 (03-08)" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5732,6 +5733,497 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: U1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 03/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>310,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>جام + كلانش أمبرطي</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>480,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>مسكة الزبل</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>موطار</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>38,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>152,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>عدس أحمر</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>18,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>تومة</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>390,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>1170,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>كرطون زنجبيل عرق</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>كلانش طاولة</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>540,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>315,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>كوفس أمبرطي</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي شوربة عربي</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>جام طاولة</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>26,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>936,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>8248,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 11 (04/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -27,6 +27,7 @@
     <sheet name="فاتورة 44" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="فاتورة U1 (02-08)" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="فاتورة U1 (03-08)" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="فاتورة 11 (04-08)" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6224,6 +6225,445 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 11</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 04/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>210,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>منسوم ها 1/2 روتوس</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>310,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>كلانش Star</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>حمص خشنة</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>750,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>قلاي دسكي</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>خل أبيض</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>8,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>96,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>ندو حرك</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>كوبايلي فرة</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr"/>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>إضافي</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>42,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>42,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr"/>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Serviette</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>4762,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 23 (05/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -28,6 +28,7 @@
     <sheet name="فاتورة U1 (02-08)" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="فاتورة U1 (03-08)" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="فاتورة 11 (04-08)" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="فاتورة 23 (05-08)" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6664,6 +6665,497 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 23</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 05/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>كنور الدجاج</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>كلانش أمبرطي</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>بنزا سنون</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>425,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>قرفة عواد</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>40,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>؟ (1×108)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>108,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>108,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>؟ (3×35)</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>؟ (4×28)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>28,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>112,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>شطابة</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>24,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>96,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>؟ (50×42)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>42,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>2100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>؟ (5×27)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>27,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>135,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>6361,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoices No. 19 (06/08) and No. 21 (07/08)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -29,6 +29,8 @@
     <sheet name="فاتورة U1 (03-08)" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="فاتورة 11 (04-08)" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="فاتورة 23 (05-08)" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="فاتورة 19 (06-08)" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="فاتورة 21 (07-08)" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7156,6 +7158,1032 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 19</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 06/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>سلبطة؟ (×42)</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>42,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>2520,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>جام طاولة</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>312,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>936,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>كلانش طاولة</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>ملح</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>سلوفان</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>420,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>576,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>كوفس أمبرطي</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي شوربة عربي</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>علب صوجي تونسية ولبن خيار</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>ليباي عجينا</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي صوجي تومة قهوة</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>560,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>560,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي علب كنانة</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>وكة موسى؟</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>10749,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 21</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 07/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>كلانش Star</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>سيسون؟</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>175,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>350,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>سكر أصفر</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>6,50</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>سكر أزرق</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>7,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>كلانش + جام أمبرطي</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>كنور</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>156,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي روتوس 1/2</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس حام</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>216,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>432,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>315,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس عادي</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>بواط صوجي تومة قهوة</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>560,00</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>560,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>5354,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 13 (08/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -31,6 +31,7 @@
     <sheet name="فاتورة 23 (05-08)" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="فاتورة 19 (06-08)" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="فاتورة 21 (07-08)" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="فاتورة 13 (08-08)" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8184,6 +8185,365 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 13</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 08/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>صاك الطوب كيس</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>185,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>555,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>بنزا أمبرطي</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>90,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>أوك</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>مسكة الزبل</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>315,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>جام أمبرطي</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>كلانش أمبرطي</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>5107,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 15 (09/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -32,6 +32,7 @@
     <sheet name="فاتورة 19 (06-08)" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="فاتورة 21 (07-08)" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="فاتورة 13 (08-08)" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="فاتورة 15 (09-08)" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8544,6 +8545,449 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 15</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 09/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>940,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>حلبت</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>310,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>زيتون</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>حمص خشنة</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>750,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>ملح</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>كنور</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>156,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>ليكات</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>موطار 2K</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>38,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>228,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>ثومة بودرة</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>60,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>بصلة بودرة</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>60,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>عدس أحمر</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>18,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>حمص</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>15,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr"/>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>توب طلاصة؟</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>4692,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Correct item name حلبت -> حليب across all sheets
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -533,6 +533,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -974,6 +975,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1136,7 +1138,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1247,6 +1249,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1365,7 +1368,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1630,6 +1633,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1682,7 +1686,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -2035,6 +2039,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2109,7 +2114,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2418,6 +2423,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2470,7 +2476,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -2779,6 +2785,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2963,7 +2970,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -3382,6 +3389,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3478,7 +3486,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -3897,6 +3905,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3949,7 +3958,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -4302,6 +4311,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4376,7 +4386,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -4815,6 +4825,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4889,7 +4900,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -5324,6 +5335,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5420,7 +5432,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -5773,6 +5785,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -5825,7 +5838,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -6264,6 +6277,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -6382,7 +6396,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -6703,6 +6717,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -6931,7 +6946,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -7194,6 +7209,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -7268,7 +7284,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -7707,6 +7723,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -7781,7 +7798,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -8220,6 +8237,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -8579,6 +8597,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -8653,7 +8672,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -9022,6 +9041,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -9052,7 +9072,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -9581,6 +9601,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -9611,7 +9632,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -10162,6 +10183,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10258,7 +10280,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -10633,6 +10655,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10685,7 +10708,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -11016,6 +11039,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -11090,7 +11114,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -11531,6 +11555,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -11583,7 +11608,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -12090,6 +12115,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -12208,7 +12234,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>حلبت</t>
+          <t>حليب</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Fix names زيتون->دانون, أوك->أوني globally; add invoice No. 17 (10/08)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -33,6 +33,7 @@
     <sheet name="فاتورة 21 (07-08)" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="فاتورة 13 (08-08)" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="فاتورة 15 (09-08)" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="فاتورة 17 (10-08)" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -674,7 +675,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1160,7 +1161,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1280,7 +1281,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1818,7 +1819,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1906,7 +1907,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -2070,7 +2071,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -2630,7 +2631,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -3212,7 +3213,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -3420,7 +3421,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -3596,7 +3597,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -3980,7 +3981,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -4364,7 +4365,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -4408,7 +4409,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -4966,7 +4967,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -5208,7 +5209,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -5454,7 +5455,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -6212,7 +6213,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -6528,7 +6529,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -6594,7 +6595,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -6792,7 +6793,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -6836,7 +6837,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -7416,7 +7417,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -7636,7 +7637,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -7974,7 +7975,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -8334,7 +8335,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -8356,7 +8357,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -8694,7 +8695,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -8999,6 +9000,255 @@
       <c r="D22" s="10" t="inlineStr">
         <is>
           <t>4692,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 17</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 10/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>أوني</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>114,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>سلوفان</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>1425,00</t>
         </is>
       </c>
     </row>
@@ -9248,7 +9498,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -9358,7 +9608,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -9654,7 +9904,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -9786,7 +10036,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -10302,7 +10552,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -10796,7 +11046,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -11202,7 +11452,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -11312,7 +11562,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>أوك</t>
+          <t>أوني</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -11806,7 +12056,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -12388,7 +12638,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>زيتون</t>
+          <t>دانون</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add invoice No. 25 (11/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -34,6 +34,7 @@
     <sheet name="فاتورة 13 (08-08)" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="فاتورة 15 (09-08)" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="فاتورة 17 (10-08)" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="فاتورة 25 (11-08)" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -534,7 +535,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -976,7 +976,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1250,7 +1249,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1634,7 +1632,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2040,7 +2037,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2424,7 +2420,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2786,7 +2781,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3390,7 +3384,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3906,7 +3899,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4312,7 +4304,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4826,7 +4817,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -5336,7 +5326,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5786,7 +5775,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -6278,7 +6266,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -6718,7 +6705,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -7210,7 +7196,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -7724,7 +7709,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -8238,7 +8222,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -8598,7 +8581,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -9257,6 +9239,541 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 25</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 11/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>ملح</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>كرطون زنجبيل</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>زيتون مقطع 5K</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>255,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>جام طاولة</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>312,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>936,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>3+3</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>كلانش + جام أمبرطي</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>480,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>كنور 10K</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>156,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>كلانش Star 2L</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>نيدو وحدة</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>420,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس عادي</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>علب كنانة</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>علب مونتوس روتوس</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>شوربة عربي مطلقين</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي علب صوجي ولبن خيار</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>7876,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -9291,7 +9808,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -9851,7 +10367,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10433,7 +10948,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10905,7 +11419,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -11289,7 +11802,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -11805,7 +12317,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -12365,7 +12876,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add invoice No. 30 (12/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -35,6 +35,7 @@
     <sheet name="فاتورة 15 (09-08)" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="فاتورة 17 (10-08)" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="فاتورة 25 (11-08)" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="فاتورة 30 (12-08)" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9774,6 +9775,541 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 30</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 12/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>كنور</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>104,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>الشاي</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>جام طاولة</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>312,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>936,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>كلانش طاولة</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>بنزا سنون 3K</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>255,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>زيتون مقطع</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>255,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>كلانش أمبرطي</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>جام أمبرطي</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>مسكة الزبل</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>كنور الدجاج</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>4K</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>قطميرة</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>200,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>قطميرة مدخنة</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>60,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>كمة الرز غزال؟</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>لحم مجمد كيس</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>علفة + جكس</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>8,00</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>5650,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 31 (13/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -36,6 +36,7 @@
     <sheet name="فاتورة 17 (10-08)" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="فاتورة 25 (11-08)" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="فاتورة 30 (12-08)" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="فاتورة 31 (13-08)" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10869,6 +10870,387 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 31</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 13/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>سكر أحمر</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>قزبر مطحون</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>كلانش Star 2K</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>أوني</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>420,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>كوفس أمبرطي</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>بسمتي 5K</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>28,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>560,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>4449,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 32 (14/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -37,6 +37,7 @@
     <sheet name="فاتورة 25 (11-08)" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="فاتورة 30 (12-08)" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="فاتورة 31 (13-08)" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="فاتورة 32 (14-08)" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11251,6 +11252,387 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 32</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 14/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>940,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>سكر أزرق</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>7,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>35,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>سلوفان</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>ألمنيوم</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>510,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>صندوق كابو؟</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>1250,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>1250,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>لون فيلي؟</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>130,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>كرطون زنجبيل عرق</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>أوني</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>4959,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 20 (15/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -38,6 +38,7 @@
     <sheet name="فاتورة 30 (12-08)" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="فاتورة 31 (13-08)" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="فاتورة 32 (14-08)" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="فاتورة 20 (15-08)" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11633,6 +11634,475 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 20</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 15/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>كلانش Star</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>كلانش أمبرطي</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>جام أمبرطي</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>ملح</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي روتوس</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>أوني</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>315,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس حام</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>216,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>432,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس عادي</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي روتوس؟</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>كرطون شوكة؟</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>390,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>1170,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي بواط 5K؟</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>550,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>550,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>7258,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 26 (16/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -39,6 +39,7 @@
     <sheet name="فاتورة 31 (13-08)" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="فاتورة 32 (14-08)" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="فاتورة 20 (15-08)" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="فاتورة 26 (16-08)" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12103,6 +12104,453 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 26</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 16/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>قزبر مطحون</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>60,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>قرفة عواد</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>لوبي</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>قهوة</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>210,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>ملح</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي مهلبية</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>114,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>أوني</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>الطحين؟</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>90,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>ليكات</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>600,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>4622,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 37 (17/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -40,6 +40,7 @@
     <sheet name="فاتورة 32 (14-08)" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="فاتورة 20 (15-08)" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="فاتورة 26 (16-08)" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="فاتورة 37 (17-08)" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12551,6 +12552,343 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 37</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 17/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>حمص خشنة كيس</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>750,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>ليكات</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>كوفس أمبرطي</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي نكي كيلو؟</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي علب كنانة</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي صوجي تومة</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>560,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>560,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي شوربة عربي</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي شوربة ملكية؟</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>525,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>576,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي كوفس تومة عرق؟</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>5726,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 27 (18/08) - quantities only, prices not on paper
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -41,6 +41,7 @@
     <sheet name="فاتورة 20 (15-08)" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="فاتورة 26 (16-08)" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="فاتورة 37 (17-08)" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="فاتورة 27 (18-08)" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12889,6 +12890,215 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 27</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 18/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>فنجي؟</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>أوني</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>كوكة حفافة؟</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>كرطون باكيت اللفوم؟</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>3Kg</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>كيلو حوت/حمض دنجال؟</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>خنشة ملح خشن</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr"/>
+      <c r="D14" s="9" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 36 (19/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -42,6 +42,7 @@
     <sheet name="فاتورة 26 (16-08)" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="فاتورة 37 (17-08)" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="فاتورة 27 (18-08)" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="فاتورة 36 (19-08)" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13099,6 +13100,519 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 36</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 19/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>قلاي دسكي</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>سكر أحمر</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>6,50</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>ألمنيوم</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>85,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>510,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>جام طاولة</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>312,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>936,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>كلانش + جام أمبرطي</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>480,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>كلانش Star 2L</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>مسكة الزبل</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>أوني</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>114,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>شطابة بالعصي</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>525,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>علب كنانة أمريكي</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>576,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>شوربة عربي مطلقين</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>اللحم؟</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>سرابيت دو كوزينة؟</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>7,00</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>7622,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 38 (20/08) page 1 of 2 (partial)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -43,6 +43,7 @@
     <sheet name="فاتورة 37 (17-08)" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="فاتورة 27 (18-08)" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="فاتورة 36 (19-08)" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="فاتورة 38 (20-08)" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13613,6 +13614,497 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 38</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 20/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>525,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>576,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>علب كنانة أمريكي</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>ليكات</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>الزيت كرطون 5L</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>حليب 4A</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>سكر ثاني؟</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>45,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>نسمة دستة</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>الشاي</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>140,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>5K</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>سكر أحمر</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>6,50</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>ملح</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>كنور الدجاج</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>336,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>كتشوب معلوبين</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>كتشوب أمبرطي كبير</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>جام أمبرطي بيضي</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>خل أبيض</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>8,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>96,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>5921,00 (صفحة 1/2 - جزئي)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 41 (21/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -44,6 +44,7 @@
     <sheet name="فاتورة 27 (18-08)" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="فاتورة 36 (19-08)" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="فاتورة 38 (20-08)" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="فاتورة 41 (21-08)" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14105,6 +14106,277 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 41</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 21/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1880,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>124,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>أكاجو</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>1250,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>1250,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>سلوفان</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>30,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>الطوب</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>125,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>4153,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 43-44 (22/08), two pages combined
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -45,6 +45,7 @@
     <sheet name="فاتورة 36 (19-08)" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="فاتورة 38 (20-08)" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="فاتورة 41 (21-08)" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="فاتورة 43-44 (22-08)" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14377,6 +14378,607 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 43-44</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 22/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>زنجبيل</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>حلقة بوجخ؟</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>جام أمبرطي</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>كلانش أمبرطي</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>كلانش طاولة</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>180,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>540,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>جام طاولة</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>312,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>936,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>كلانش Star</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>708,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>أوني</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>مسكة الزبل</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>كرطون زنجبيل</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>275,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>بوز غزال</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>شوكة كرطون</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>390,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>1170,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>خنشة حمص 2K</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>750,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>كنور 10K</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>104,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>10K</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>مسكة بيضاء</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>40,00</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>سكر أحمر</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>6,50</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>32,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>420,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس عادي</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>9528,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add invoice No. 45 (23/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -46,6 +46,7 @@
     <sheet name="فاتورة 38 (20-08)" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="فاتورة 41 (21-08)" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="فاتورة 43-44 (22-08)" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="فاتورة 45 (23-08)" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15560,6 +15561,431 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 45</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 23/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>186,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>نسمة 2K</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>كلانش Star 2L</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>25,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>150,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>مسكة الزبل</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>315,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>384,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>شوربة أمبرطي عربي</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>شوربة مطلقين</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>360,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>كوفس أمبرطي</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>ليباي</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>12,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>120,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي علب كنانة</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>375,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>ملعقة Star</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>6,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>18,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>5034,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Correct item name كلانش/كتشوب -> كاتشب (ketchup) across all sheets
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -547,6 +547,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -988,6 +989,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1084,7 +1086,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>كلانش أمبرطمي</t>
+          <t>كاتشب أمبرطمي</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1106,7 +1108,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>كلانش 24</t>
+          <t>كاتشب 24</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1261,6 +1263,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1357,7 +1360,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>كلانش Star</t>
+          <t>كاتشب Star</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1423,7 +1426,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>كلانش أ مبرطمي</t>
+          <t>كاتشب أ مبرطمي</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1644,6 +1647,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2049,6 +2053,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2145,7 +2150,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>كلانش Star</t>
+          <t>كاتشب Star</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -2432,6 +2437,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2528,7 +2534,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>كلانش أ مبرطمي</t>
+          <t>كاتشب أ مبرطمي</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -2793,6 +2799,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3021,7 +3028,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>كلانش Star</t>
+          <t>كاتشب Star</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -3285,7 +3292,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>كلانش طابة</t>
+          <t>كاتشب طابة</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -3396,6 +3403,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3756,7 +3764,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>كلانش أ مبرطي</t>
+          <t>كاتشب أ مبرطي</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -3911,6 +3919,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4051,7 +4060,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>كلانش أ مبرطي</t>
+          <t>كاتشب أ مبرطي</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -4316,6 +4325,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4829,6 +4839,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4925,7 +4936,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>كلانش Star 24</t>
+          <t>كاتشب Star 24</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -5123,7 +5134,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>كلانش + جام أمبرطي</t>
+          <t>كاتشب + جام أمبرطي</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -5338,6 +5349,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5566,7 +5578,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>كلانش 24</t>
+          <t>كاتشب 24</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -5787,6 +5799,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -5861,7 +5874,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>جام + كلانش أمبرطي</t>
+          <t>جام + كاتشب أمبرطي</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -6037,7 +6050,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>كلانش طاولة</t>
+          <t>كاتشب طاولة</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -6278,6 +6291,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -6418,7 +6432,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>كلانش Star</t>
+          <t>كاتشب Star</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -6717,6 +6731,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -6857,7 +6872,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>كلانش أمبرطي</t>
+          <t>كاتشب أمبرطي</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -7208,6 +7223,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -7348,7 +7364,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>كلانش طاولة</t>
+          <t>كاتشب طاولة</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -7721,6 +7737,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -7773,7 +7790,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>كلانش Star</t>
+          <t>كاتشب Star</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -7993,7 +8010,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>كلانش + جام أمبرطي</t>
+          <t>كاتشب + جام أمبرطي</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -8234,6 +8251,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -8528,7 +8546,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>كلانش أمبرطي</t>
+          <t>كاتشب أمبرطي</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -8593,6 +8611,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -9036,6 +9055,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -9285,6 +9305,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -9513,7 +9534,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>كلانش + جام أمبرطي</t>
+          <t>كاتشب + جام أمبرطي</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -9557,7 +9578,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>كلانش Star 2L</t>
+          <t>كاتشب Star 2L</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -9820,6 +9841,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -10004,7 +10026,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>كلانش طاولة</t>
+          <t>كاتشب طاولة</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -10092,7 +10114,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>كلانش أمبرطي</t>
+          <t>كاتشب أمبرطي</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -10355,6 +10377,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10693,7 +10716,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>كلانش سطاريط</t>
+          <t>كاتشب سطاريط</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -10914,6 +10937,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -11032,7 +11056,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>كلانش Star 2K</t>
+          <t>كاتشب Star 2K</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -11295,6 +11319,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -11676,6 +11701,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -11728,7 +11754,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>كلانش Star</t>
+          <t>كاتشب Star</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -11772,7 +11798,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>كلانش أمبرطي</t>
+          <t>كاتشب أمبرطي</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -12145,6 +12171,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12592,6 +12619,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12929,6 +12957,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -13138,6 +13167,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -13300,7 +13330,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>كلانش + جام أمبرطي</t>
+          <t>كاتشب + جام أمبرطي</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -13322,7 +13352,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>كلانش Star 2L</t>
+          <t>كاتشب Star 2L</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -13651,6 +13681,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -13989,7 +14020,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>كتشوب معلوبين</t>
+          <t>كاتشب معلوبين</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -14011,7 +14042,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>كتشوب أمبرطي كبير</t>
+          <t>كاتشب أمبرطي كبير</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -14142,6 +14173,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -14413,6 +14445,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -14553,7 +14586,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>كلانش أمبرطي</t>
+          <t>كاتشب أمبرطي</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -14575,7 +14608,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>كلانش طاولة</t>
+          <t>كاتشب طاولة</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -14619,7 +14652,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>كلانش Star</t>
+          <t>كاتشب Star</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -15014,6 +15047,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -15242,7 +15276,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>كلانش أ مبرطمي</t>
+          <t>كاتشب أ مبرطمي</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -15595,6 +15629,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -15713,7 +15748,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>كلانش Star 2L</t>
+          <t>كاتشب Star 2L</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -16020,6 +16055,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -16204,7 +16240,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>كلانش 24</t>
+          <t>كاتشب 24</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -16491,6 +16527,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -16565,7 +16602,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>كلانش أ مبرطمي</t>
+          <t>كاتشب أ مبرطمي</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -16874,6 +16911,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -17389,6 +17427,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -17507,7 +17546,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>كلانش بسكري كبيرة</t>
+          <t>كاتشب بسكري كبيرة</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -17859,7 +17898,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>جام أمبرطمي + كلانش أ مبرطمي</t>
+          <t>جام أمبرطمي + كاتشب أ مبرطمي</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -17948,6 +17987,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add invoice No. 51 (24/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -47,6 +47,7 @@
     <sheet name="فاتورة 41 (21-08)" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="فاتورة 43-44 (22-08)" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="فاتورة 45 (23-08)" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="فاتورة 51 (24-08)" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +548,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -989,7 +989,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1263,7 +1262,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1647,7 +1645,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2053,7 +2050,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2437,7 +2433,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2799,7 +2794,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3403,7 +3397,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3919,7 +3912,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4325,7 +4317,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4839,7 +4830,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -5349,7 +5339,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5799,7 +5788,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -6291,7 +6279,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -6731,7 +6718,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -7223,7 +7209,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -7737,7 +7722,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -8251,7 +8235,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -8611,7 +8594,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -9055,7 +9037,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -9305,7 +9286,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -9841,7 +9821,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -10377,7 +10356,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10937,7 +10915,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -11319,7 +11296,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -11701,7 +11677,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12171,7 +12146,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12619,7 +12593,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12957,7 +12930,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -13167,7 +13139,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -13681,7 +13652,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -14173,7 +14143,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -14445,7 +14414,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -15047,7 +15015,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -15629,7 +15596,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -16013,6 +15979,431 @@
       <c r="D21" s="10" t="inlineStr">
         <is>
           <t>5034,50</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 51</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 24/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>ملعقة</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>40,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>قرفة موسى؟</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>70,00</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>210,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>كاتشب أمبرطي</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>320,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>جام أمبرطي بيضي</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>النشا</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>خمسة حبوب؟</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>96,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>96,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>خنشة سمسم محمر</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>400,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>400,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>حبة موداعا؟</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>80,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>160,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>بنزا أبيض</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>130,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>260,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>الطماطم عائشة</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>29,50</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>354,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>ماس أبيض كيس؟</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>185,00</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>370,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>ماس أبيض صغير؟</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>315,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>جافيل</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>19,00</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>57,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>4499,50</t>
         </is>
       </c>
     </row>
@@ -16055,7 +16446,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -16527,7 +16917,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -16911,7 +17300,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -17427,7 +17815,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -17987,7 +18374,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add invoice No. 52 (25/08) as a separate sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HUo2BJA8p6j7Z1kUJr8agN
</commit_message>
<xml_diff>
--- a/فاتورة_أبطال_الشام.xlsx
+++ b/فاتورة_أبطال_الشام.xlsx
@@ -48,6 +48,7 @@
     <sheet name="فاتورة 43-44 (22-08)" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="فاتورة 45 (23-08)" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="فاتورة 51 (24-08)" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="فاتورة 52 (25-08)" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16412,6 +16413,365 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أبطال الشام</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>فاتورة رقم: 52</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ: 25/08/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>نوع البضاعة</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>الثمن</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>الزيت</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>470,00</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1410,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>حليب</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>62,00</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>248,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>نسمة</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>10,50</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>94,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>كنور الدجاج</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>168,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>دانون</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>2,50</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>75,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>ملح</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>20,00</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>40,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>قندري 25</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>112,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>كنور 10K</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>52,00</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>156,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي علب كنانة كبير 3K</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>450,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>سربيت</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>105,00</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>525,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>كلانكس</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>192,00</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>576,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي علب جوخ تومة بلبن</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>أمبرطي نصف كيلو روتوس</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>300,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>المجموع</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>4805,00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>